<commit_message>
Param-agnostic next-page detection (not hardcoded to ?p=/?page=)
Replaces the brittle "?p=/page=" anchor match with a layered, param-name-agnostic
next-page detector: profile next_page selector -> rel=next -> next-labelled anchors
(text/aria/class) -> same-path numeric query-param increment (catches ?p, ?page, ?x,
?start, ?offset, ?pg, ...) -> path-based (page-2.html, /page/2). Restricted to the
same host (+ same path for query pagination), which also fixes a cross-domain
false-positive (an external dentallearning.net link was being treated as "next").

Note (verified): Safco returns the same first 15 products in static HTML regardless of
?page=N — its pagination is client-side JS — so this detector still can't reach Safco
page 2 via httpx; that needs the Playwright tier. Demonstrated working on books.toscrape.

8 new navigate tests (each param style + cross-domain exclusion). 27 total, all green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/books_demo/products.xlsx
+++ b/data/books_demo/products.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311918+00:00</t>
+          <t>2026-06-27T04:50:02.486907+00:00</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568733+00:00</t>
+          <t>2026-06-27T04:50:00.310366+00:00</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195923+00:00</t>
+          <t>2026-06-27T04:50:01.406969+00:00</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195894+00:00</t>
+          <t>2026-06-27T04:50:01.406951+00:00</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196093+00:00</t>
+          <t>2026-06-27T04:50:01.407161+00:00</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195874+00:00</t>
+          <t>2026-06-27T04:50:01.406933+00:00</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195857+00:00</t>
+          <t>2026-06-27T04:50:01.406915+00:00</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195840+00:00</t>
+          <t>2026-06-27T04:50:01.406897+00:00</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195821+00:00</t>
+          <t>2026-06-27T04:50:01.406877+00:00</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195801+00:00</t>
+          <t>2026-06-27T04:50:01.406854+00:00</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195764+00:00</t>
+          <t>2026-06-27T04:50:01.406807+00:00</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196077+00:00</t>
+          <t>2026-06-27T04:50:01.407143+00:00</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569135+00:00</t>
+          <t>2026-06-27T04:50:00.310744+00:00</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569120+00:00</t>
+          <t>2026-06-27T04:50:00.310728+00:00</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196063+00:00</t>
+          <t>2026-06-27T04:50:01.407127+00:00</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569105+00:00</t>
+          <t>2026-06-27T04:50:00.310710+00:00</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569089+00:00</t>
+          <t>2026-06-27T04:50:00.310694+00:00</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569072+00:00</t>
+          <t>2026-06-27T04:50:00.310677+00:00</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196048+00:00</t>
+          <t>2026-06-27T04:50:01.407112+00:00</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311892+00:00</t>
+          <t>2026-06-27T04:50:02.486888+00:00</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311863+00:00</t>
+          <t>2026-06-27T04:50:02.486865+00:00</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569057+00:00</t>
+          <t>2026-06-27T04:50:00.310660+00:00</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568889+00:00</t>
+          <t>2026-06-27T04:50:00.310493+00:00</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569040+00:00</t>
+          <t>2026-06-27T04:50:00.310644+00:00</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569025+00:00</t>
+          <t>2026-06-27T04:50:00.310628+00:00</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.569010+00:00</t>
+          <t>2026-06-27T04:50:00.310613+00:00</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568869+00:00</t>
+          <t>2026-06-27T04:50:00.310473+00:00</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311814+00:00</t>
+          <t>2026-06-27T04:50:02.486824+00:00</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196033+00:00</t>
+          <t>2026-06-27T04:50:01.407096+00:00</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568846+00:00</t>
+          <t>2026-06-27T04:50:00.310453+00:00</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568995+00:00</t>
+          <t>2026-06-27T04:50:00.310597+00:00</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196018+00:00</t>
+          <t>2026-06-27T04:50:01.407082+00:00</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568979+00:00</t>
+          <t>2026-06-27T04:50:00.310582+00:00</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568962+00:00</t>
+          <t>2026-06-27T04:50:00.310566+00:00</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568946+00:00</t>
+          <t>2026-06-27T04:50:00.310546+00:00</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568927+00:00</t>
+          <t>2026-06-27T04:50:00.310529+00:00</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196003+00:00</t>
+          <t>2026-06-27T04:50:01.407066+00:00</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195989+00:00</t>
+          <t>2026-06-27T04:50:01.407051+00:00</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195973+00:00</t>
+          <t>2026-06-27T04:50:01.407034+00:00</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.315426+00:00</t>
+          <t>2026-06-27T04:50:02.489494+00:00</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.315400+00:00</t>
+          <t>2026-06-27T04:50:02.489478+00:00</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3454,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.315372+00:00</t>
+          <t>2026-06-27T04:50:02.489461+00:00</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568909+00:00</t>
+          <t>2026-06-27T04:50:00.310512+00:00</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.315326+00:00</t>
+          <t>2026-06-27T04:50:02.489442+00:00</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312208+00:00</t>
+          <t>2026-06-27T04:50:02.489417+00:00</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312184+00:00</t>
+          <t>2026-06-27T04:50:02.487098+00:00</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312162+00:00</t>
+          <t>2026-06-27T04:50:02.487082+00:00</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312137+00:00</t>
+          <t>2026-06-27T04:50:02.487065+00:00</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:48.568817+00:00</t>
+          <t>2026-06-27T04:50:00.310427+00:00</t>
         </is>
       </c>
     </row>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312114+00:00</t>
+          <t>2026-06-27T04:50:02.487049+00:00</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312091+00:00</t>
+          <t>2026-06-27T04:50:02.487033+00:00</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312065+00:00</t>
+          <t>2026-06-27T04:50:02.487016+00:00</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312042+00:00</t>
+          <t>2026-06-27T04:50:02.486999+00:00</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.312018+00:00</t>
+          <t>2026-06-27T04:50:02.486981+00:00</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195956+00:00</t>
+          <t>2026-06-27T04:50:01.407013+00:00</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311994+00:00</t>
+          <t>2026-06-27T04:50:02.486964+00:00</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311970+00:00</t>
+          <t>2026-06-27T04:50:02.486946+00:00</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:50.311944+00:00</t>
+          <t>2026-06-27T04:50:02.486927+00:00</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.195940+00:00</t>
+          <t>2026-06-27T04:50:01.406997+00:00</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>2026-06-27T04:25:49.196107+00:00</t>
+          <t>2026-06-27T04:50:01.407182+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>